<commit_message>
Streamline UI, add in-page evaluation report, remove Neon DB text, and update agile methodology records
</commit_message>
<xml_diff>
--- a/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
@@ -617,12 +617,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>FastAPI /api/chat returns 500 error when question payload is empty or whitespace</t>
+          <t>POST /api/evaluate endpoint returned 500 when request payload omitted the ai_response field</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -642,12 +642,12 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Added request input validation and raised HTTP 400 Bad Request with descriptive message</t>
+          <t>Added Pydantic Field validation with required constraint and descriptive 400 Bad Request error response</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Verified with empty string and whitespace test cases</t>
+          <t>Verified with empty string and missing field test cases</t>
         </is>
       </c>
     </row>
@@ -672,12 +672,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>SQuAD dataset load failure on Python 3.13 due to dataclass type mismatch in Hugging Face library</t>
+          <t>Hugging Face datasets library threw ArrowTypeError when loading SQuAD validation split on Python 3.13</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Switched dataset loader to canonical squad validation split and selected 1000 sample subset</t>
+          <t>Switched to canonical squad validation split and parsed question-context pairs directly into standard dictionary format</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Successfully extracted 1,000 QA contexts without schema errors</t>
+          <t>Extracted 1,000 QA context pairs without schema errors</t>
         </is>
       </c>
     </row>
@@ -727,12 +727,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Windows cp1252 terminal console encoding error when printing non-ASCII characters from ingested text</t>
+          <t>PyTorch and TensorFlow DLL collision on Windows caused Python process crash during sentence-transformers embedding generation</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -747,17 +747,17 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Maintainability</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Sanitized console text preview outputs using ascii encoding fallback with replacement</t>
+          <t>Configured USE_TF=0 and USE_TORCH=1 environment variables before importing sentence-transformers</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Prevents terminal crash during ingestion progress logging</t>
+          <t>Resolved C++ runtime lockup on Windows</t>
         </is>
       </c>
     </row>
@@ -782,12 +782,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>AI generated markdown formatting displaying raw asterisks in response card</t>
+          <t>PyMuPDF text extraction failed with unhandled exception when processing empty or scan-only PDF pages</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -802,17 +802,17 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>User Interface</t>
+          <t>Logical</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Implemented inline markdown parser to render bold text and bullet points cleanly</t>
+          <t>Added text length check per page with fallback warning if extracted text is empty</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Verified bold response rendering in browser</t>
+          <t>Prevents pipeline crash on blank document pages</t>
         </is>
       </c>
     </row>
@@ -837,12 +837,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>RAG pipeline execution spinner remained spinning after all retrieval steps completed</t>
+          <t>Frontend evaluation pipeline progress indicator remained spinning after backend returned evaluation verdict</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Updated step completion condition to display static checkmark when pipeline reaches final step</t>
+          <t>Updated pipeline state check to transition step indicator to static checkmark on step 6 completion</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Progress indicator transitions cleanly to completed state</t>
+          <t>Progress bar transitions cleanly to 100% completed state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
align 2x2 overview grid, improve ui visibility, enhance hallucination statement flags, and update sprint 2 agile files
</commit_message>
<xml_diff>
--- a/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
@@ -882,69 +882,279 @@
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="6" t="n"/>
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Relevance Judge score occasionally exceeded 5.0 boundary or returned float with excessive decimal places</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Clamped score with min(5.0, max(1.0, raw_score)) and rounded to 1 decimal place</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Verified score remains strictly between 1.0 and 5.0 across varied queries</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Accuracy Agent incorrectly marked out-of-domain questions as PASS by hallucinating facts from general LLM pretraining</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Added strict closed-world grounding check returning Insufficient Evidence / Unverified when grounding chunks are empty</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Verified out-of-domain query returns UNVERIFIED status with notice banner</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="6" t="n"/>
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Gemini API returned 404 NotFound on deprecated gemini-2.0-flash model causing validation pipeline failure</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Updated primary model to gemini-3.6-flash and added multi-model fallback across 3.7-flash and 3.1-flash-lite</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Resolved model deprecation with seamless fallback</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="6" t="n"/>
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>All 4 Overview tab cards rendered with uneven heights and staggered alignment due to column wrapping</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Replaced staggered column wrappers with direct 2x2 CSS Grid using grid-auto-rows: 1fr and equal stretch</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>All 4 overview boxes render with identical height and clean symmetry</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Hallucination Agent only flagged entire response without breaking down individual unsupported or fabricated statements</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Added statement-by-statement extraction with Supported, Unsupported, Fabricated, and Contradictory classifications</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Each claim displays distinct highlight badge, cited evidence, and violation reason</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="5" t="n"/>

</xml_diff>

<commit_message>
docs(agile): update sprint 3 methodology files, defect tracker, and test plan
</commit_message>
<xml_diff>
--- a/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
@@ -1157,82 +1157,334 @@
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="6" t="n"/>
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Completeness Agent failed to penalize partially addressed multi-part questions when AI response used conversational filler</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Updated prompt with specific omission breakdown and negative constraint checking against query clauses</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Verified with multi-part science and history test questions</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Verdict Agent composite score displayed IEEE 754 floating point precision anomalies in UI summary</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Rounded composite score to 2 decimal places in backend verdict_agent.py and applied safeScore formatting in frontend</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Weighted score renders cleanly as 4.33 / 5.00</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="6" t="n"/>
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>CSV Batch upload failed silently when file contained empty trailing rows or unescaped comma characters</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Added csv.Sniffer dialect detection, non-empty row filtering, and strip whitespace preprocessing in parse_csv</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Successfully parses CSV files with blank lines and commas in text fields</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Analytics Dashboard KPI cards displayed NaN when database had zero evaluation records in selected date range</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Added null-coalescing defaults (0 count, 0.0 avg score) and empty-state guidance illustrations</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard renders zero-state gracefully without calculation errors</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="6" t="n"/>
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Inspect modal triggered unhandled JavaScript TypeError (.map is not a function) when inspecting records during active batch evaluation</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Added safeList, safeScore, and safeParseJson helpers, parsed DB JSON strings, and wrapped modal in InspectErrorBoundary</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Inspect modal opens cleanly without screen blanking even during active batch runs</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="6" t="n"/>
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Evaluation pipeline latency reached 90 seconds due to 429 quota exhaustion and 20s gRPC retry loops on gemini-3.6-flash</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Switched PRIMARY_MODEL to gemini-3.1-flash-lite, configured dual API key rotation, and set request timeouts</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Evaluation latency reduced from 90s to 5.18s with all 5 independent agents intact</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="5" t="n"/>

</xml_diff>

<commit_message>
feat: SentryAI rebranding, inspect modal UI polish, analytics fix, and agile methodology update
</commit_message>
<xml_diff>
--- a/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Defects" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="125725" fullCalcOnLoad="1"/>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="17.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -1487,43 +1487,334 @@
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="6" t="n"/>
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Radar chart label text on left and right axes ('Completeness', 'Accuracy') clipped at outer edge of SVG container</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Expanded radar viewBox to 390x270, centered radarCx to 195, and offset label coordinates with textAnchor alignment</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Verified labels render with ample margin on both 1366px and 1920px displays</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Donut chart verdict distribution legend descriptions truncated prematurely with CSS text-overflow ellipsis</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Rebalanced flex ratios, removed restrictive max-width constraint, and crafted concise status descriptions</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Full text visible for all 4 verdict categories without trailing ellipsis</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="6" t="n"/>
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Batch evaluation Inspect modal exhibited horizontal scrollbar and rendered raw stringified JSON dictionaries for verified and flagged claims</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Replaced JSON.stringify with structured claim cards, added formatAspectText helper, set grid minmax(0, 1fr), and set overflow-x: hidden</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>Modal displays formatted cards with badges and sources; zero horizontal scroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>API rate limits encountered during heavy consecutive batch evaluations when relying strictly on single LLM provider free-tier quota</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Integrated OpenAI GPT-4o-mini provider fallback alongside Gemini key rotation with unified response adapter</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Batch runs fail over seamlessly without hitting 429 quota exhaustion</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Batch evaluation PDF report lacked granular question-by-question breakdown table with individual agent scores</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Enhanced report_generator.py to build multi-page tables listing question excerpts, agent scores, composite, and final verdicts</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>PDF export generates comprehensive audit report with executive KPIs and itemized details</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Global branding inconsistency across browser title, top navigation, sidebar, and favicon prior to final presentation</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Rebranded platform to SentryAI, updated HTML titles, headers, footers, and replaced default Vite icon with custom SentryAI shield/iris SVG</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Unified SentryAI identity active across all browser surfaces and reports</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(milestone4): complete analytics filters, executive PDF reports, agile tracking, and benchmark datasets
</commit_message>
<xml_diff>
--- a/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="17.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -1813,6 +1813,166 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>Unified SentryAI identity active across all browser surfaces and reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Analytics Dashboard threw 500 Internal Server Error when selecting Pass/Fail verdict filters due to unescaped % character in psycopg2 SQL query</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Refactored SQL query in get_analytics_summary to use parameterized LIKE %s placeholders with tuple params</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Batch, Verdict, and Model Engine dropdowns in Analytics Dashboard rendered with unstyled OS native dropdown controls and white option menus</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Restyled filter bar with custom glassmorphic pill cards, SVG chevrons, theme-consistent dark option backgrounds, and active border glow</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Analytics Model Engine filter did not separate OpenAI and Gemini evaluation results because model selection was not persisted as a dedicated database column</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Logical</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Added ai_engine VARCHAR(64) column to evaluation_records and batch_evaluations tables and updated save_evaluation and create_batch_job</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Single and Batch PDF reports lacked dynamic total page numbering (Page X of Y) and running header on subsequent pages</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Nitin Patel</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>User Interface</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Implemented custom NumberedCanvas class in report_generator.py to calculate two-pass page counts and render running headers and footers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(agile): add MIT license, complete agile templates, and close defects for final submission
- Add MIT License (LICENSE) and reference badge in README.md
- Update Defect_Tracker Template_v0.1.xlsx to close defects 23-26 with action dates and resolution remarks
- Update Agile_Template_v0.1.xls: distribute Sprint 3 and Sprint 4 day-wise task hours in Sprint Backlog; add US_30 and US_31 to Product and Sprint Backlog
- Update Unit_Test_Plan_v0.1.xlsx: add UT_33 verifying MIT license and open-source compliance
</commit_message>
<xml_diff>
--- a/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_methodologyFiles/Defect_Tracker Template_v0.1.xlsx
@@ -1855,6 +1855,21 @@
           <t>Refactored SQL query in get_analytics_summary to use parameterized LIKE %s placeholders with tuple params</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Parameterized queries active; verified zero SQL exceptions across all verdict filters</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1895,6 +1910,21 @@
           <t>Restyled filter bar with custom glassmorphic pill cards, SVG chevrons, theme-consistent dark option backgrounds, and active border glow</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Custom styled glassmorphism dropdowns active with SVG icons and dark theme styling</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1935,6 +1965,21 @@
           <t>Added ai_engine VARCHAR(64) column to evaluation_records and batch_evaluations tables and updated save_evaluation and create_batch_job</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ai_engine column added to schema; per-model filtering fully operational</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1973,6 +2018,21 @@
       <c r="H27" t="inlineStr">
         <is>
           <t>Implemented custom NumberedCanvas class in report_generator.py to calculate two-pass page counts and render running headers and footers</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>NumberedCanvas two-pass page numbering and running headers verified across all PDF reports</t>
         </is>
       </c>
     </row>

</xml_diff>